<commit_message>
feat(claims): expand Claims Portal test suite to 40 TCs covering mobile views, FAQ mutex, tooltips, and file management
</commit_message>
<xml_diff>
--- a/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
+++ b/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1624,9 +1624,415 @@
         <v>Figma Frame 630 (Functional Specifications &amp; Rules)</v>
       </c>
     </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>TC-GW-CLM-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Mobile Responsiveness</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Claims Listing Mobile Layout (375px)</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Verify Mobile View Layout for My Claims Listing (375px Viewport)</v>
+      </c>
+      <c r="F32" t="str">
+        <v>User views claims portal on mobile device (375px viewport).</v>
+      </c>
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Set viewport to 375x812
+2. Navigate to My Claims
+3. Inspect layout hierarchy, compact table, and navigation selector.</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Renders mobile layout per Frame 2383-11615: top compact account selector [ My Claims ⌵ ], compact 5-column table (Order, Date, Total, Status, Actions), full-width search input above horizontal scrolling status tabs, full-width [ CREATE NEW CLAIM ] button.</v>
+      </c>
+      <c r="I32" t="str">
+        <v>BLOCKED: 302 Redirect loop to My Dashboard on mobile.</v>
+      </c>
+      <c r="J32" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K32" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Figma Frame 2383-11615 (mobile/my_account/My Claims)</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>TC-GW-CLM-032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Mobile Responsiveness</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Create Claim Mobile Layout (375px)</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Verify Mobile View Layout for Create Claim Form (375px Viewport)</v>
+      </c>
+      <c r="F33" t="str">
+        <v>User accesses claim creation on mobile device.</v>
+      </c>
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Set viewport to 375x812
+2. Navigate to /claims/create
+3. Verify form fields, dropzone, and CTAs stacking.</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Renders mobile form per Frame 2383-11131: single-column vertically stacked fields, full-width file dropzone, full-width stacked action buttons [ REVIEW ] and [ BACK ].</v>
+      </c>
+      <c r="I33" t="str">
+        <v>BLOCKED: Returns HTTP 404 Not Found.</v>
+      </c>
+      <c r="J33" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K33" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Figma Frame 2383-11131 (mobile/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>TC-GW-CLM-033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>FAQ Accordion Block</v>
+      </c>
+      <c r="C34" t="str">
+        <v>FAQ Mutex &amp; Admin Rule</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Verify FAQ Block Mutex Behavior and Max 8 Accordions Rule</v>
+      </c>
+      <c r="F34" t="str">
+        <v>User on My Claims or Create Claim page viewing FAQ block.</v>
+      </c>
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Count rendered FAQ accordion items (max 8)
+2. Verify all accordions closed by default
+3. Click to open Accordion 1
+4. Click to open Accordion 2
+5. Verify Accordion 1 closes automatically.</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Up to 8 FAQs rendered; closed by default; strict mutex behavior enforced (opening an accordion closes previously opened accordion) per Frame 630.</v>
+      </c>
+      <c r="I34" t="str">
+        <v>BLOCKED: Portal undeployed.</v>
+      </c>
+      <c r="J34" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K34" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Figma Frame 630 (Functional Specifications &amp; Rules)</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>TC-GW-CLM-034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>UI Table Behavior</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Action Column Display Logic</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Verify Action Column Displays Direct 'VIEW' Link vs Dropdown (Frame 630 Rule)</v>
+      </c>
+      <c r="F35" t="str">
+        <v>User viewing claims grid.</v>
+      </c>
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect row with only 'VIEW' action available
+2. Inspect row with multiple actions (e.g., View, Upload Documents, Cancel)
+3. Verify UI presentation.</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Per Frame 630: If 'VIEW' is the only action, hide the dropdown wrapper and render 'VIEW' as a direct inline link. If multiple actions exist, house them inside an actions dropdown.</v>
+      </c>
+      <c r="I35" t="str">
+        <v>BLOCKED: Claims listing inaccessible.</v>
+      </c>
+      <c r="J35" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K35" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Figma Frame 630 (Functional Specifications &amp; Rules)</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>TC-GW-CLM-035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>UI Table Behavior</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Order Number Hyperlink Navigation</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Verify Order Number is Clickable Hyperlink to Order Details</v>
+      </c>
+      <c r="F36" t="str">
+        <v>User viewing claims list containing order reference numbers.</v>
+      </c>
+      <c r="G36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect Order Number cell (e.g. #CH03021)
+2. Verify element is an anchor tag with href pointing to /sales/order/view/order_id/...
+3. Click Order link and verify navigation.</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Per Frame 630: Order Number is an interactive clickable hyperlink navigating directly to that order's detail page.</v>
+      </c>
+      <c r="I36" t="str">
+        <v>BLOCKED: Claims listing inaccessible.</v>
+      </c>
+      <c r="J36" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K36" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Figma Frame 630 (Functional Specifications &amp; Rules)</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>TC-GW-CLM-036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>UI Table Behavior</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Pagination Controls &amp; Item Counter</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Verify Pagination Controls and Items Counter per Frame 630</v>
+      </c>
+      <c r="F37" t="str">
+        <v>User has more claims than the configured items-per-page limit.</v>
+      </c>
+      <c r="G37" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect bottom of claims table
+2. Verify item count display on the left (e.g. 'X items')
+3. Verify page switcher on the right ([ 1 ] [ 2 ] [ &gt; ])
+4. Click next page and verify grid update.</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Renders pagination bar per Frame 630: counter on left, page switcher on right, backend-configurable items per page.</v>
+      </c>
+      <c r="I37" t="str">
+        <v>BLOCKED: Claims listing inaccessible.</v>
+      </c>
+      <c r="J37" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K37" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Figma Frame 630 (Functional Specifications &amp; Rules)</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>TC-GW-CLM-037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Create Claim Form</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Help Tooltips (🛈)</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Verify Interactive Help Tooltips on Form Fields per Frame 631</v>
+      </c>
+      <c r="F38" t="str">
+        <v>User on Create Claim form.</v>
+      </c>
+      <c r="G38" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate tooltips on: 'Claim type', 'Product or Invoice No', 'Quantity', 'Preferred resolution', 'Description of issue'
+2. Hover/click each tooltip
+3. Verify contextual helper popover appears with admin-configured text.</v>
+      </c>
+      <c r="H38" t="str">
+        <v>All 5 specified fields feature interactive 🛈 tooltips with administrative copy per Frame 631 &amp; Frame 2383-11003.</v>
+      </c>
+      <c r="I38" t="str">
+        <v>BLOCKED: Create Claim form returns 404.</v>
+      </c>
+      <c r="J38" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K38" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Figma Frame 631 (Create Claim Functional Specifications)</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>TC-GW-CLM-038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Create Claim Form</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Media Dropzone &amp; File Removal</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Verify Media Upload Thumbnail Rendering and File Deletion Action</v>
+      </c>
+      <c r="F39" t="str">
+        <v>User uploads valid images (.jpg, .png) or video (.mp4, .mov) under 100MB.</v>
+      </c>
+      <c r="G39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Upload 2 files to dropzone
+2. Verify thumbnail previews and filenames render
+3. Click [ DELETE ] button on file 1
+4. Verify file 1 is removed from upload queue while file 2 remains.</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Thumbnails render dynamically alongside uploaded file names; [ DELETE ] action cleanly removes individual files prior to submission per Frame 2383-11003.</v>
+      </c>
+      <c r="I39" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J39" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K39" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>TC-GW-CLM-039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Create Claim Form</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Preferred Resolution Selection</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Verify Preferred Resolution Dropdown Options and Selection</v>
+      </c>
+      <c r="F40" t="str">
+        <v>User filling Create Claim form.</v>
+      </c>
+      <c r="G40" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Preferred resolution' dropdown
+2. Inspect available options
+3. Select an option (e.g., Replacement, Credit, Repair)
+4. Verify selected option persists.</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Dropdown provides standardized resolution options (Replacement, Credit Note, Repair, Refund) per Figma Frame 2383-11003.</v>
+      </c>
+      <c r="I40" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J40" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K40" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>TC-GW-CLM-040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Create Claim Workflow</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Review Summary &amp; Form Progression</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Verify Form Progression: [ REVIEW ] Summary Step and [ BACK ] State Preservation</v>
+      </c>
+      <c r="F41" t="str">
+        <v>User has filled all required claim form fields.</v>
+      </c>
+      <c r="G41" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click [ REVIEW ] button
+2. Verify system displays Claim Summary review modal/page
+3. Click [ BACK ] button
+4. Verify user returns to edit form with all entered data, attached photos, and selections intact.</v>
+      </c>
+      <c r="H41" t="str">
+        <v>[ REVIEW ] navigates to summary review before lodging; [ BACK ] returns to form preserving all user input without data loss per Figma Frame 2383-11003 &amp; Frame 631.</v>
+      </c>
+      <c r="I41" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J41" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K41" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Figma Frame 631 &amp; Frame 2383-11003</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(claims): expand test suite to 50 comprehensive TCs covering empty states, search debounce, quantity bounds, file limits, and confirmation
</commit_message>
<xml_diff>
--- a/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
+++ b/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2030,9 +2030,412 @@
         <v>Figma Frame 631 &amp; Frame 2383-11003</v>
       </c>
     </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>TC-GW-CLM-041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>UI Table States</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Empty State Handling</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Verify Empty State Display When No Claims Exist for Selected Filter</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Account with zero claims or filter returning 0 records.</v>
+      </c>
+      <c r="G42" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to My Claims with empty account or filter with 0 items
+2. Inspect table container
+3. Verify empty state copy and action CTA.</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Renders clean empty state ('You have no claims in this view') with primary [ CREATE NEW CLAIM ] CTA button; no broken table or JavaScript error per Frame 2383-11454.</v>
+      </c>
+      <c r="I42" t="str">
+        <v>BLOCKED: 302 Redirect loop to My Dashboard.</v>
+      </c>
+      <c r="J42" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K42" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Figma Frame 2383-11454 (desktop/my_account/My Claims)</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>TC-GW-CLM-042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Claims Search &amp; Filtering</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Table Search Bar</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Verify Live Keyword Search Filtering Across Claims Table</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Customer has multiple claims across different orders/products.</v>
+      </c>
+      <c r="G43" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter keyword in search input (e.g. Order #, SKU, or Product Name)
+2. Observe table update without page reload
+3. Clear search bar.</v>
+      </c>
+      <c r="H43" t="str">
+        <v>System dynamically filters table rows matching search query with debounce (300ms) without full page reload per Frame 2383-11454.</v>
+      </c>
+      <c r="I43" t="str">
+        <v>BLOCKED: Claims listing inaccessible.</v>
+      </c>
+      <c r="J43" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K43" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Figma Frame 2383-11454 (desktop/my_account/My Claims)</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>TC-GW-CLM-043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Claims Search &amp; Filtering</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Status Filter Tabs (ALL, OPEN, PENDING, CLOSED)</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Verify Status Filter Tab Switching and Active Indicator</v>
+      </c>
+      <c r="F44" t="str">
+        <v>User on My Claims listing page.</v>
+      </c>
+      <c r="G44" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'ALL' tab
+2. Click 'OPEN' tab
+3. Click 'PENDING' tab
+4. Click 'CLOSED' tab
+5. Verify active tab styling and URL/state update.</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Tab switches active indicator (underline/pill), updates displayed claims instantly or via clean AJAX request, and preserves filter state per Frame 2383-11454.</v>
+      </c>
+      <c r="I44" t="str">
+        <v>BLOCKED: Route redirects to Dashboard.</v>
+      </c>
+      <c r="J44" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K44" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Figma Frame 2383-11454 (desktop/my_account/My Claims)</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>TC-GW-CLM-044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Navigation &amp; Hierarchy</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Sidebar Active Indicator (AGENTS.md Rule 2)</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Verify My Account Sidebar 'MY CLAIMS' Active Brown Pill Styling and Sub-Items</v>
+      </c>
+      <c r="F45" t="str">
+        <v>User viewing any Claims view.</v>
+      </c>
+      <c r="G45" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect My Account left navigation sidebar
+2. Inspect 'MY CLAIMS' menu item
+3. Check computed background color, border-radius, and sub-items (Open Claims, Pending Claims, Closed Claims).</v>
+      </c>
+      <c r="H45" t="str">
+        <v>'MY CLAIMS' item renders active brown pill styling with sub-items expanded per Figma Frame 2383-11454 and Rule 2 of AGENTS.md.</v>
+      </c>
+      <c r="I45" t="str">
+        <v>BLOCKED: Inaccessible on live storefront (302 redirect).</v>
+      </c>
+      <c r="J45" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K45" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Figma Frame 2383-11454 (desktop/my_account/My Claims)</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>TC-GW-CLM-045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Form Validation</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Quantity Bound Enforcement</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Verify Claim Quantity Cannot Exceed Purchased Invoice Quantity</v>
+      </c>
+      <c r="F46" t="str">
+        <v>User selected product with invoice quantity of 2.</v>
+      </c>
+      <c r="G46" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate Quantity field
+2. Attempt to input quantity higher than invoice quantity (e.g., 5)
+3. Attempt to proceed to Review.</v>
+      </c>
+      <c r="H46" t="str">
+        <v>System enforces quantity constraint: field max value locked to purchased quantity or shows inline error 'Quantity cannot exceed purchased quantity (2)' per Frame 2383-11003.</v>
+      </c>
+      <c r="I46" t="str">
+        <v>BLOCKED: Create Claim form undeployed (404).</v>
+      </c>
+      <c r="J46" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K46" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
+        <v>TC-GW-CLM-046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Media Intake Validation</v>
+      </c>
+      <c r="C47" t="str">
+        <v>File Size Limit (100MB)</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Verify Rejection of Media Files Exceeding 100MB Limit</v>
+      </c>
+      <c r="F47" t="str">
+        <v>User attempts to upload file &gt; 100MB.</v>
+      </c>
+      <c r="G47" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a video or image file &gt; 100MB (e.g. 110MB .mp4)
+2. Drop into upload dropzone
+3. Verify upload rejection.</v>
+      </c>
+      <c r="H47" t="str">
+        <v>System blocks file with clear validation toast/error: 'File size exceeds maximum limit of 100MB' per Frame 2383-11003 &amp; Frame 631.</v>
+      </c>
+      <c r="I47" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J47" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K47" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Figma Frame 631 (Create Claim Functional Specifications)</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
+        <v>TC-GW-CLM-047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Media Intake Validation</v>
+      </c>
+      <c r="C48" t="str">
+        <v>File Extension Whitelist</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Verify Rejection of Disallowed File Extensions (.pdf, .exe, .zip)</v>
+      </c>
+      <c r="F48" t="str">
+        <v>User attempts to upload non-supported media type.</v>
+      </c>
+      <c r="G48" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Attempt to upload a .pdf or .zip file
+2. Drop into file dropzone
+3. Verify validation error.</v>
+      </c>
+      <c r="H48" t="str">
+        <v>System strictly enforces allowed formats (.jpg, .png, .mp4, .mov) and rejects other formats with 'Unsupported file type' error per Frame 2383-11003.</v>
+      </c>
+      <c r="I48" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J48" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K48" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
+        <v>TC-GW-CLM-048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Submission &amp; Notifications</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Confirmation Screen &amp; Email Trigger</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Verify Post-Submission Confirmation Screen and Automated Email Trigger</v>
+      </c>
+      <c r="F49" t="str">
+        <v>User successfully submits a complete claim.</v>
+      </c>
+      <c r="G49" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Complete review step and click [ SUBMIT CLAIM ]
+2. Verify confirmation page renders
+3. Verify display of NetSuite Case ID and timeline expectation
+4. Verify automated email dispatch.</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Page renders confirmation banner with NetSuite Case Number, resolution SLA details, and dispatches confirmation email to customer email address per Frame 2383-11003 &amp; Frame 630.</v>
+      </c>
+      <c r="I49" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J49" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K49" t="str">
+        <v>P0 - CRITICAL</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Figma Frame 630 &amp; Frame 2383-11003</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
+        <v>TC-GW-CLM-049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Dual-Auth Matrix</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Logged-Out Public Browsing Mode (AGENTS.md Rule 3)</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Logged-Out / Guest User</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Verify Unauthenticated Guest Access to Claims URL Redirects to Login with Referer</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Guest user browsing storefront without logging in.</v>
+      </c>
+      <c r="G50" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open incognito/guest browser
+2. Navigate directly to https://mcstaging2.globewest.com/claims
+3. Verify HTTP status and redirection.</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Unauthenticated users are redirected cleanly to /customer/account/login/ with referer parameter (or 404 masked); wholesale portal is strictly inaccessible per Rule 3 of AGENTS.md.</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Pass: Guest cannot access authenticated claims data.</v>
+      </c>
+      <c r="J50" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="K50" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L50" t="str">
+        <v>AGENTS.md Dual-Auth Matrix</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
+        <v>TC-GW-CLM-050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Dual-Auth Matrix &amp; AU Baseline</v>
+      </c>
+      <c r="C51" t="str">
+        <v>AU Storefront Anti-Regression Safeguard (AGENTS.md Rule 3)</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Authenticated (AU Customer / Trade deepalilondhe576@gmail.com)</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Verify AU Baseline Storefront Invariant Integrity (Zero Defect Leakage from US Scope)</v>
+      </c>
+      <c r="F51" t="str">
+        <v>User authenticated on AU Staging (https://mcstaging2.globewest.com.au).</v>
+      </c>
+      <c r="G51" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Login with AU credentials (deepalilondhe576@gmail.com / Deep@123)
+2. Navigate to AU My Account
+3. Verify AU claims architecture remains unchanged without US experimental route leakage.</v>
+      </c>
+      <c r="H51" t="str">
+        <v>AU storefront operates on established baseline without regressions, broken redirects, or US theme leakage per Rule 3 of AGENTS.md.</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Pass: AU baseline intact.</v>
+      </c>
+      <c r="J51" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="K51" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L51" t="str">
+        <v>AGENTS.md Dual-Auth Matrix &amp; AU Baseline</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(claims): expand test suite to 55 TCs, verify clean spacing, and set custom Excel column widths
</commit_message>
<xml_diff>
--- a/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
+++ b/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
@@ -397,7 +397,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L56"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="35.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="7" max="7" width="65.83203125" customWidth="1"/>
+    <col min="8" max="8" width="60.83203125" customWidth="1"/>
+    <col min="9" max="9" width="55.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="45.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2433,9 +2447,209 @@
         <v>AGENTS.md Dual-Auth Matrix &amp; AU Baseline</v>
       </c>
     </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
+        <v>TC-GW-CLM-051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Search &amp; Claim Creation</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Autocomplete Suggestions Dropdown</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Verify Product Search Autocomplete Dropdown Renders Product Name, SKU, PO Number, and Invoice Number</v>
+      </c>
+      <c r="F52" t="str">
+        <v>User on Create Claim form entering characters in the search field.</v>
+      </c>
+      <c r="G52" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Type partial product name (e.g. 'Pearce') in search field
+2. Wait for suggestion dropdown to appear
+3. Verify metadata displayed for each matching suggestion.</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Live dropdown renders matching items showing Product Name, SKU, Customer PO Number, and Invoice Number for quick selection per Figma Frame 2383-11003 &amp; Frame 631.</v>
+      </c>
+      <c r="I52" t="str">
+        <v>BLOCKED: Create Claim form undeployed (HTTP 404).</v>
+      </c>
+      <c r="J52" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K52" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Figma Frame 2383-11003 &amp; Frame 631</v>
+      </c>
+    </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53" t="str">
+        <v>TC-GW-CLM-052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Search &amp; Claim Creation</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Autocomplete Empty Result Feedback</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Verify Search Autocomplete Displays 'No Matching Purchased Products Found' for Non-Purchased Items</v>
+      </c>
+      <c r="F53" t="str">
+        <v>User searches for a product or SKU never purchased by this trade account.</v>
+      </c>
+      <c r="G53" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter a non-purchased SKU or random product title
+2. Observe autocomplete dropdown area
+3. Verify messaging and absence of broken errors.</v>
+      </c>
+      <c r="H53" t="str">
+        <v>System gracefully displays informational feedback: 'No matching purchased products or invoices found' without crashing per Figma Frame 2383-11003.</v>
+      </c>
+      <c r="I53" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J53" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K53" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54" t="str">
+        <v>TC-GW-CLM-053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Create Claim Workflow</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Multi-Product Claims Management</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Verify Removal of Individual Product Item from Multi-Product Claim Submission</v>
+      </c>
+      <c r="F54" t="str">
+        <v>User added two products to a single claim using '+ ADD ANOTHER PRODUCT'.</v>
+      </c>
+      <c r="G54" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate second product item card in claim form
+2. Click '[ REMOVE ITEM ]' link / button
+3. Verify product 2 is removed while product 1 remains intact.</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Selected product is removed cleanly from the claim package; remaining product fields and form state persist without page reload per Frame 2383-11003.</v>
+      </c>
+      <c r="I54" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J54" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K54" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55" t="str">
+        <v>TC-GW-CLM-054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Form Validation</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Mandatory Fields Inline Validation</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Verify Inline Red Border and Validation Error Messages for All Mandatory Fields on Empty Submit</v>
+      </c>
+      <c r="F55" t="str">
+        <v>User on Create Claim page with all fields blank.</v>
+      </c>
+      <c r="G55" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Leave all fields empty
+2. Click '[ REVIEW ]' button
+3. Verify error indicators on: Claim type, Product/Invoice, Quantity, Preferred resolution, Description, and Photo upload.</v>
+      </c>
+      <c r="H55" t="str">
+        <v>All empty mandatory fields receive red border outline and explicit contextual error copy (e.g. 'This is a required field', 'Minimum one photo required') per Frame 2383-11003 &amp; Frame 631.</v>
+      </c>
+      <c r="I55" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J55" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K55" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Figma Frame 631 (Create Claim Functional Specifications)</v>
+      </c>
+    </row>
+    <row r="56" xml:space="preserve">
+      <c r="A56" t="str">
+        <v>TC-GW-CLM-055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Need Help &amp; Support Block</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Help Centre CTA on Create Claim Page</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Verify Create Claim 'Questions about your claim?' Block and 'VISIT HELP CENTRE' Navigation</v>
+      </c>
+      <c r="F56" t="str">
+        <v>User viewing bottom section of Create Claim page.</v>
+      </c>
+      <c r="G56" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Scroll to 'Questions about your claim?' block
+2. Verify copy and '[ VISIT HELP CENTRE ]' button
+3. Click button and verify clean navigation to Help Centre URL without 404.</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Help block renders per Frame 2383-11003; button links to valid US Help Centre route with verified contact options.</v>
+      </c>
+      <c r="I56" t="str">
+        <v>BLOCKED: Create Claim page undeployed (404).</v>
+      </c>
+      <c r="J56" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K56" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(claims): expand test suite to 60 comprehensive TCs covering WCAG accessibility, debounce, drag-and-drop, and network resilience
</commit_message>
<xml_diff>
--- a/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
+++ b/Sprint-3/Ticket_Claims_Portal/Claims_Portal_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L61"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2647,9 +2647,209 @@
         <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
       </c>
     </row>
+    <row r="57" xml:space="preserve">
+      <c r="A57" t="str">
+        <v>TC-GW-CLM-056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Accessibility &amp; Usability</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Keyboard Navigation (WCAG 2.1 AA)</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Verify Keyboard Focus Order and Interactive Tab Traversal Across Create Claim Form</v>
+      </c>
+      <c r="F57" t="str">
+        <v>User on Create Claim page using keyboard only.</v>
+      </c>
+      <c r="G57" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Press Tab key sequentially from top of page
+2. Verify focus moves logically through Claim Type, Product Lookup, Quantity, Resolution, Description, Dropzone, and Review CTA
+3. Verify visible high-contrast focus rings on all inputs.</v>
+      </c>
+      <c r="H57" t="str">
+        <v>Tab order follows logical DOM reading hierarchy without keyboard traps; all inputs feature visible focus states meeting WCAG 2.1 AA standards per Frame 2383-11003.</v>
+      </c>
+      <c r="I57" t="str">
+        <v>BLOCKED: Create Claim form undeployed (404).</v>
+      </c>
+      <c r="J57" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K57" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Figma Frame 2383-11003 &amp; Frame 631</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
+      <c r="A58" t="str">
+        <v>TC-GW-CLM-057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Media Intake Validation</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Drag-and-Drop Active States</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Verify Drag-and-Drop Active Visual Hover Feedback on Media Dropzone</v>
+      </c>
+      <c r="F58" t="str">
+        <v>User dragging media files from local operating system.</v>
+      </c>
+      <c r="G58" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Drag valid image file over upload dropzone container
+2. Observe dropzone visual styling while file is hovered
+3. Release file to trigger upload.</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Dropzone triggers active dragover state with highlighted border (#381C12) and helper copy change ('Drop files here to upload') per Frame 2383-11003.</v>
+      </c>
+      <c r="I58" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J58" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K58" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="L58" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="59" xml:space="preserve">
+      <c r="A59" t="str">
+        <v>TC-GW-CLM-058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Submission &amp; Notifications</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Double-Submission Debounce</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Verify Rapid Double-Click Debounce Prevention on Claim Submission CTA</v>
+      </c>
+      <c r="F59" t="str">
+        <v>User on final Claim Review step ready to submit.</v>
+      </c>
+      <c r="G59" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Rapidly click '[ SUBMIT CLAIM ]' button twice within 300ms
+2. Verify button state immediately after first click
+3. Verify only one NetSuite case record is created.</v>
+      </c>
+      <c r="H59" t="str">
+        <v>Button is immediately disabled with inline spinner upon initial click; secondary click is ignored, preventing duplicate NetSuite Case IDs per Frame 630 &amp; Frame 631.</v>
+      </c>
+      <c r="I59" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J59" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K59" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L59" t="str">
+        <v>Figma Frame 630 &amp; Frame 631</v>
+      </c>
+    </row>
+    <row r="60" xml:space="preserve">
+      <c r="A60" t="str">
+        <v>TC-GW-CLM-059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Form Validation</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Special Characters &amp; XSS Sanitization</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Verify Special Characters, Emojis, and HTML Sanitization in Issue Description</v>
+      </c>
+      <c r="F60" t="str">
+        <v>User entering complex text in Description textarea.</v>
+      </c>
+      <c r="G60" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter text with emojis ('📦 Damaged leg &amp; scratch ⚡'), quotes, and HTML tags ('&lt;script&gt;alert(1)&lt;/script&gt;')
+2. Submit claim
+3. Inspect rendered summary and NetSuite ticket.</v>
+      </c>
+      <c r="H60" t="str">
+        <v>Textarea accepts multiline formatting and emojis cleanly; HTML/script tags are safely sanitized to prevent XSS and database corruption per Frame 2383-11003.</v>
+      </c>
+      <c r="I60" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J60" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K60" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L60" t="str">
+        <v>Figma Frame 2383-11003 (desktop/my_account/Create Claim)</v>
+      </c>
+    </row>
+    <row r="61" xml:space="preserve">
+      <c r="A61" t="str">
+        <v>TC-GW-CLM-060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Network &amp; Error Resilience</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Backend API &amp; Timeout Handling</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Authenticated (US Trade Customer)</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Verify Graceful Error Recovery Banner on Backend API or NetSuite Timeout</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Network latency or backend NetSuite gateway timeout during submission.</v>
+      </c>
+      <c r="G61" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Simulate 504 Gateway Timeout or network drop during claim submit
+2. Observe UI response
+3. Verify user does not lose entered form data.</v>
+      </c>
+      <c r="H61" t="str">
+        <v>System displays non-disruptive error alert: 'We are currently unable to submit your claim. Please retry or contact support' while preserving all entered form data for easy re-try per Frame 630.</v>
+      </c>
+      <c r="I61" t="str">
+        <v>BLOCKED: Form undeployed (404).</v>
+      </c>
+      <c r="J61" t="str">
+        <v>FAIL (Blocked by P0)</v>
+      </c>
+      <c r="K61" t="str">
+        <v>P1 - HIGH</v>
+      </c>
+      <c r="L61" t="str">
+        <v>Figma Frame 630 (Functional Specifications &amp; Rules)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>